<commit_message>
12 Mitarbeiter und echte Praxiszeiten von Ida-Sophie Kranz & Kollegen
Mitarbeiter: 3 Zahnärztinnen, 2 Prophylaxeassistentinnen, 1 Dentalhygienikerin,
3 ZFA, 2 Verwaltungsassistentinnen, 1 Abrechnungshelferin.

Öffnungszeiten: Mo/Do 08-13+14-18, Di 08-15+16-20, Mi/Fr 08-13.
Excel enthält neue Öffnungszeiten-Spalte und Legende je Wochentag.

https://claude.ai/code/session_019fWqJA8pFyvjYkpdvVzAbU
</commit_message>
<xml_diff>
--- a/dienstplan_2025-06.xlsx
+++ b/dienstplan_2025-06.xlsx
@@ -62,12 +62,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -114,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -126,8 +126,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -135,7 +141,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -504,23 +510,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="5" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Dienstplan Juni 2025 – Zahnarztpraxis</t>
+          <t>Dienstplan Juni 2025 – Ida-Sophie Kranz &amp; Kollegen, Essen  |  Mo/Do: 08-13+14-18  |  Di: 08-15+16-20  |  Mi/Fr: 08-13</t>
         </is>
       </c>
     </row>
@@ -542,27 +556,67 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Öffnungszeit</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Dr. Schmidt</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Dr. Müller</t>
-        </is>
-      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Dr. Hoffmann</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Wagner</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Sandra Becker</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Miriam Schulz</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Petra Lange</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
           <t>Anna Weber</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Lisa Braun</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Tanja Fischer</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Jana Koch</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Maria Richter</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Sabine Klein</t>
         </is>
       </c>
     </row>
@@ -582,7 +636,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -601,6 +655,46 @@
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -622,25 +716,65 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
+          <t>08:00–13:00 / 14:00–18:00</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N4" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O4" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P4" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -662,25 +796,65 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
+          <t>08:00–15:00 / 16:00–20:00</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P5" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -702,27 +876,67 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
+          <t>08:00–13:00</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
         </is>
       </c>
     </row>
@@ -742,25 +956,65 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
+          <t>08:00–13:00 / 14:00–18:00</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -782,27 +1036,67 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
+          <t>08:00–13:00</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
         </is>
       </c>
     </row>
@@ -822,7 +1116,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -841,6 +1135,46 @@
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -862,7 +1196,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -881,6 +1215,46 @@
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -902,25 +1276,65 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
+          <t>08:00–13:00 / 14:00–18:00</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P11" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -942,25 +1356,65 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
+          <t>08:00–15:00 / 16:00–20:00</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O12" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P12" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -982,27 +1436,67 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
+          <t>08:00–13:00</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="M13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P13" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
         </is>
       </c>
     </row>
@@ -1022,25 +1516,65 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
+          <t>08:00–13:00 / 14:00–18:00</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -1062,27 +1596,67 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
+          <t>08:00–13:00</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1676,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1121,6 +1695,46 @@
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -1142,7 +1756,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1161,6 +1775,46 @@
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -1182,25 +1836,65 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
+          <t>08:00–13:00 / 14:00–18:00</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -1222,25 +1916,65 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
+          <t>08:00–15:00 / 16:00–20:00</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -1262,27 +1996,67 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
+          <t>08:00–13:00</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="N20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="O20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P20" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
         </is>
       </c>
     </row>
@@ -1302,25 +2076,65 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
+          <t>08:00–13:00 / 14:00–18:00</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P21" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -1342,27 +2156,67 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
+          <t>08:00–13:00</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="M22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="O22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
         </is>
       </c>
     </row>
@@ -1382,7 +2236,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -1401,6 +2255,46 @@
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="P23" s="4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -1422,7 +2316,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -1441,6 +2335,46 @@
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -1462,25 +2396,65 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
+          <t>08:00–13:00 / 14:00–18:00</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N25" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O25" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P25" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -1502,25 +2476,65 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
+          <t>08:00–15:00 / 16:00–20:00</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L26" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M26" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N26" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O26" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P26" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -1542,27 +2556,67 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
+          <t>08:00–13:00</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="M27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="N27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="O27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P27" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
         </is>
       </c>
     </row>
@@ -1582,25 +2636,65 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
+          <t>08:00–13:00 / 14:00–18:00</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L28" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M28" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N28" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O28" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P28" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -1622,27 +2716,67 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
+          <t>08:00–13:00</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="M29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="N29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="O29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P29" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
         </is>
       </c>
     </row>
@@ -1662,7 +2796,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1681,6 +2815,46 @@
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="P30" s="4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -1702,7 +2876,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -1721,6 +2895,46 @@
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="P31" s="4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -1742,25 +2956,65 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
+          <t>08:00–13:00 / 14:00–18:00</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="L32" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M32" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="N32" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="O32" s="7" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="P32" s="7" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -1768,7 +3022,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1780,58 +3034,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Statistik Juni 2025</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Rolle</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>Ganztag</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>Vormittag</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="10" t="inlineStr">
         <is>
           <t>Nachmittag</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="10" t="inlineStr">
         <is>
           <t>Urlaub</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="10" t="inlineStr">
         <is>
           <t>Krankheit</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="10" t="inlineStr">
         <is>
           <t>Frei</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="10" t="inlineStr">
         <is>
           <t>Arbeitstage</t>
         </is>
@@ -1849,10 +3103,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -1873,19 +3127,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dr. Müller</t>
+          <t>Dr. Hoffmann</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Zahnarzt</t>
+          <t>Zahnärztin</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -1906,19 +3160,19 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Anna Weber</t>
+          <t>Dr. Wagner</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ZFA</t>
+          <t>Zahnärztin</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -1939,19 +3193,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Lisa Braun</t>
+          <t>Sandra Becker</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ZFA</t>
+          <t>Prophylaxeassistentin</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -1972,19 +3226,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jana Koch</t>
+          <t>Miriam Schulz</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empfang</t>
+          <t>Prophylaxeassistentin</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -1999,6 +3253,237 @@
         <v>9</v>
       </c>
       <c r="I7" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Petra Lange</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dentalhygienikerin</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>13</v>
+      </c>
+      <c r="D8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>9</v>
+      </c>
+      <c r="I8" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Anna Weber</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ZFA</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>13</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>9</v>
+      </c>
+      <c r="I9" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Lisa Braun</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ZFA</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D10" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>9</v>
+      </c>
+      <c r="I10" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tanja Fischer</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ZFA</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>9</v>
+      </c>
+      <c r="I11" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Jana Koch</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Verwaltungsassistentin</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>13</v>
+      </c>
+      <c r="D12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>9</v>
+      </c>
+      <c r="I12" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Maria Richter</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Verwaltungsassistentin</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>13</v>
+      </c>
+      <c r="D13" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>9</v>
+      </c>
+      <c r="I13" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sabine Klein</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Abrechnungshelferin</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>13</v>
+      </c>
+      <c r="D14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>9</v>
+      </c>
+      <c r="I14" t="n">
         <v>21</v>
       </c>
     </row>
@@ -2013,18 +3498,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Schichtcodes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>V</t>
         </is>
@@ -2036,82 +3521,149 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>variabel je Tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Nachmittag</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>variabel je Tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ganztag</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>V + N kombiniert</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Urlaub</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Krankheit</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Frei</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Öffnungszeiten</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Montag</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:00–13:00 und 14:00–18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Dienstag</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:00–15:00 und 16:00–20:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Mittwoch</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>08:00–13:00</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Nachmittag</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>14:00–18:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Ganztag</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>08:00–18:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Urlaub</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Krankheit</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Frei</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Donnerstag</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:00–13:00 und 14:00–18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Freitag</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08:00–13:00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>